<commit_message>
Fix login/signup retry-after-error, add Kommentar to Excel import/export
Login and signup used uncontrolled inputs. After a Server Action
returned an error (wrong password, duplicate email), a second click
on submit silently did nothing — no request, no error, just stuck —
until the page was reloaded. Next.js dispatches Server Actions one at
a time per client, and that sequential dispatch doesn't reliably pick
up a retried submission from uncontrolled fields. Switching both
forms' inputs to controlled state fixes it; verified the exact
duplicate-email and wrong-password retry paths now work.

Kommentar was missing from the Excel import, export, and downloadable
template entirely — added to all three, and to the getFilteredCatches
query the export route reads from (it wasn't selecting the column).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/fangst-mall.xlsx
+++ b/public/fangst-mall.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>Art</t>
   </si>
@@ -31,6 +31,9 @@
     <t>Bete</t>
   </si>
   <si>
+    <t>Kommentar</t>
+  </si>
+  <si>
     <t>Datum</t>
   </si>
   <si>
@@ -44,6 +47,9 @@
   </si>
   <si>
     <t>Wobbler</t>
+  </si>
+  <si>
+    <t>Tog på fallande vatten</t>
   </si>
 </sst>
 </file>
@@ -428,7 +434,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -436,10 +442,11 @@
     <col min="3" max="3" width="11" customWidth="1"/>
     <col min="4" max="5" width="16" customWidth="1"/>
     <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="12" customWidth="1"/>
+    <col min="7" max="7" width="24" customWidth="1"/>
+    <col min="8" max="8" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -461,10 +468,13 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B2">
         <v>75</v>
@@ -473,15 +483,18 @@
         <v>3.2</v>
       </c>
       <c r="D2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G2" s="2">
+        <v>11</v>
+      </c>
+      <c r="G2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H2" s="2">
         <v>46187.91666666667</v>
       </c>
     </row>

</xml_diff>